<commit_message>
feat: initialize project structure with Next.js setup, global styles, and base API routes.
</commit_message>
<xml_diff>
--- a/Tareas.xlsx
+++ b/Tareas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\repositorios_github\TFM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D724E9AD-C38C-4969-A21F-E01E76C6D1A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89CFA1A3-63AE-4B46-A502-9D8EA941D069}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{851AC7AC-0C01-4AA1-B918-0B3E26E4D0FB}"/>
+    <workbookView xWindow="11970" yWindow="2145" windowWidth="23745" windowHeight="17340" xr2:uid="{851AC7AC-0C01-4AA1-B918-0B3E26E4D0FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
feat: add documentation management module with document and database schema configuration features
</commit_message>
<xml_diff>
--- a/Tareas.xlsx
+++ b/Tareas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\repositorios_github\TFM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89CFA1A3-63AE-4B46-A502-9D8EA941D069}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AE146D8-06D0-4535-911B-8D0F36663077}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11970" yWindow="2145" windowWidth="23745" windowHeight="17340" xr2:uid="{851AC7AC-0C01-4AA1-B918-0B3E26E4D0FB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{851AC7AC-0C01-4AA1-B918-0B3E26E4D0FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="53">
   <si>
     <t>Marcel</t>
   </si>
@@ -195,6 +195,13 @@
   </si>
   <si>
     <t>Front End</t>
+  </si>
+  <si>
+    <t>Reunion
+04/06/26</t>
+  </si>
+  <si>
+    <t>done</t>
   </si>
 </sst>
 </file>
@@ -266,7 +273,10 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="11">
+  <dxfs count="12">
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -320,21 +330,22 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B1F80A3B-4E7F-41E9-A313-57DFEF224AD9}" name="Tabla1" displayName="Tabla1" ref="A1:I18" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
-  <autoFilter ref="A1:I18" xr:uid="{B1F80A3B-4E7F-41E9-A313-57DFEF224AD9}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B1F80A3B-4E7F-41E9-A313-57DFEF224AD9}" name="Tabla1" displayName="Tabla1" ref="A1:J18" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
+  <autoFilter ref="A1:J18" xr:uid="{B1F80A3B-4E7F-41E9-A313-57DFEF224AD9}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G18">
     <sortCondition ref="G1:G18"/>
   </sortState>
-  <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{589D6F3F-C9C4-48C2-A152-BD2659727C79}" name="Tarea Principal" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{6482FBAC-6B56-4B6B-B068-6C3D45EE5D84}" name="Descripcion" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{37F21341-8E00-41BB-96AC-C8A74C5A5803}" name="Asignado" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{402E759D-82A7-40F9-8C46-D0A9E28AD693}" name="Prioridad" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{BAF9ECD1-B8D1-4253-9212-0CCD4259CB7A}" name="Profesor" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{70DB6CCF-A12F-4453-BF64-CF18C52DE295}" name="Columna1" dataDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{5942CD9E-292C-4439-954F-6249C3117470}" name="Reunion_x000a_15/05/26" dataDxfId="2"/>
-    <tableColumn id="8" xr3:uid="{52D8F1E7-3147-4E9A-AA03-B18F48FABAC5}" name="Reunion_x000a_18/05/2025" dataDxfId="1"/>
-    <tableColumn id="9" xr3:uid="{8B279CE7-51C9-432D-8876-19D3A3878842}" name="Reunion_x000a_26/05/26" dataDxfId="0"/>
+  <tableColumns count="10">
+    <tableColumn id="1" xr3:uid="{589D6F3F-C9C4-48C2-A152-BD2659727C79}" name="Tarea Principal" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{6482FBAC-6B56-4B6B-B068-6C3D45EE5D84}" name="Descripcion" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{37F21341-8E00-41BB-96AC-C8A74C5A5803}" name="Asignado" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{402E759D-82A7-40F9-8C46-D0A9E28AD693}" name="Prioridad" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{BAF9ECD1-B8D1-4253-9212-0CCD4259CB7A}" name="Profesor" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{70DB6CCF-A12F-4453-BF64-CF18C52DE295}" name="Columna1" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{5942CD9E-292C-4439-954F-6249C3117470}" name="Reunion_x000a_15/05/26" dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{52D8F1E7-3147-4E9A-AA03-B18F48FABAC5}" name="Reunion_x000a_18/05/2025" dataDxfId="2"/>
+    <tableColumn id="9" xr3:uid="{8B279CE7-51C9-432D-8876-19D3A3878842}" name="Reunion_x000a_26/05/26" dataDxfId="1"/>
+    <tableColumn id="10" xr3:uid="{1ED3DD2D-B85A-4B69-9924-8E01CFC3CA08}" name="Reunion_x000a_04/06/26" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -657,7 +668,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{865E27E8-88FF-4631-B4E1-D37537FD837A}">
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.140625" customWidth="1"/>
@@ -667,9 +678,10 @@
     <col min="5" max="5" width="11.42578125" style="4"/>
     <col min="6" max="6" width="4.5703125" style="7" customWidth="1"/>
     <col min="7" max="8" width="11.42578125" style="4" customWidth="1"/>
+    <col min="10" max="10" width="12.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>2</v>
       </c>
@@ -697,8 +709,11 @@
       <c r="I1" s="8" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" s="1" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J1" s="8" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" s="1" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
@@ -724,8 +739,11 @@
       <c r="I2" s="8" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" s="1" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J2" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" s="1" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -749,8 +767,11 @@
       <c r="I3" s="8">
         <v>46172</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" s="1" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J3" s="5">
+        <v>46208</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" s="1" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>39</v>
       </c>
@@ -774,8 +795,11 @@
       <c r="I4" s="8">
         <v>46172</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J4" s="5">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>26</v>
       </c>
@@ -801,8 +825,11 @@
       <c r="I5" s="8" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J5" s="8" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>20</v>
       </c>
@@ -826,8 +853,11 @@
       <c r="I6" s="8" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J6" s="8" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>27</v>
       </c>
@@ -853,8 +883,11 @@
       <c r="I7" s="2" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J7" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>15</v>
       </c>
@@ -878,8 +911,11 @@
       <c r="I8" s="8">
         <v>46178</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J8" s="5">
+        <v>46183</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>9</v>
       </c>
@@ -905,8 +941,11 @@
       <c r="I9" s="8">
         <v>46178</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J9" s="5">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
@@ -930,8 +969,11 @@
       <c r="I10" s="8">
         <v>46173</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J10" s="5">
+        <v>46183</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>37</v>
       </c>
@@ -955,8 +997,11 @@
       <c r="I11" s="5">
         <v>46183</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J11" s="5">
+        <v>46183</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>48</v>
       </c>
@@ -980,8 +1025,11 @@
       <c r="I12" s="5">
         <v>46171</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J12" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>21</v>
       </c>
@@ -1005,8 +1053,11 @@
       <c r="I13" s="8">
         <v>46173</v>
       </c>
-    </row>
-    <row r="14" spans="1:9" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J13" s="5">
+        <v>46188</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>50</v>
       </c>
@@ -1030,8 +1081,11 @@
       <c r="I14" s="5">
         <v>46183</v>
       </c>
-    </row>
-    <row r="15" spans="1:9" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J14" s="5">
+        <v>46188</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>28</v>
       </c>
@@ -1057,8 +1111,11 @@
       <c r="I15" s="8">
         <v>46178</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J15" s="5">
+        <v>46185</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>23</v>
       </c>
@@ -1082,8 +1139,11 @@
       <c r="I16" s="8">
         <v>46183</v>
       </c>
-    </row>
-    <row r="17" spans="1:9" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J16" s="5">
+        <v>46188</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>35</v>
       </c>
@@ -1109,8 +1169,11 @@
       <c r="I17" s="8">
         <v>46188</v>
       </c>
-    </row>
-    <row r="18" spans="1:9" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J17" s="5">
+        <v>46193</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>3</v>
       </c>
@@ -1134,8 +1197,11 @@
       <c r="I18" s="8">
         <v>46193</v>
       </c>
-    </row>
-    <row r="19" spans="1:9" ht="41.25" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="J18" s="5">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="41.25" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>